<commit_message>
Corrige quebras de pagina e area de impressao da planilha de etiquetas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KBPpToZFjBagAJeWDfvD5H
</commit_message>
<xml_diff>
--- a/etiquetas-oficiais.xlsx
+++ b/etiquetas-oficiais.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etiquetas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Etiquetas'!$A$1:$B$84</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Etiquetas'!$A$1:$B$145</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="81.75" customHeight="1">
+    <row r="85" ht="113.45" customHeight="1">
       <c r="A85" s="1" t="inlineStr">
         <is>
           <t>H167</t>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="81.75" customHeight="1">
+    <row r="86" ht="113.45" customHeight="1">
       <c r="A86" s="1" t="inlineStr">
         <is>
           <t>H169</t>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="81.75" customHeight="1">
+    <row r="87" ht="113.45" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
         <is>
           <t>H171</t>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="81.75" customHeight="1">
+    <row r="88" ht="113.45" customHeight="1">
       <c r="A88" s="1" t="inlineStr">
         <is>
           <t>H173</t>
@@ -1503,7 +1503,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="81.75" customHeight="1">
+    <row r="89" ht="113.45" customHeight="1">
       <c r="A89" s="1" t="inlineStr">
         <is>
           <t>H175</t>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="81.75" customHeight="1">
+    <row r="90" ht="113.45" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
         <is>
           <t>H177</t>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="81.75" customHeight="1">
+    <row r="91" ht="113.45" customHeight="1">
       <c r="A91" s="1" t="inlineStr">
         <is>
           <t>H179</t>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="81.75" customHeight="1">
+    <row r="92" ht="113.45" customHeight="1">
       <c r="A92" s="1" t="inlineStr">
         <is>
           <t>H181</t>
@@ -1551,7 +1551,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="81.75" customHeight="1">
+    <row r="93" ht="113.45" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
         <is>
           <t>H183</t>
@@ -1563,7 +1563,7 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="81.75" customHeight="1">
+    <row r="94" ht="113.45" customHeight="1">
       <c r="A94" s="1" t="inlineStr">
         <is>
           <t>H185</t>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="81.75" customHeight="1">
+    <row r="95" ht="113.45" customHeight="1">
       <c r="A95" s="1" t="inlineStr">
         <is>
           <t>H187</t>
@@ -1587,7 +1587,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="81.75" customHeight="1">
+    <row r="96" ht="113.45" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
         <is>
           <t>H189</t>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="81.75" customHeight="1">
+    <row r="97" ht="113.45" customHeight="1">
       <c r="A97" s="1" t="inlineStr">
         <is>
           <t>H191</t>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="81.75" customHeight="1">
+    <row r="98" ht="113.45" customHeight="1">
       <c r="A98" s="1" t="inlineStr">
         <is>
           <t>H193</t>
@@ -1623,7 +1623,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="81.75" customHeight="1">
+    <row r="99" ht="113.45" customHeight="1">
       <c r="A99" s="1" t="inlineStr">
         <is>
           <t>H195</t>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="81.75" customHeight="1">
+    <row r="100" ht="113.45" customHeight="1">
       <c r="A100" s="1" t="inlineStr">
         <is>
           <t>H197</t>
@@ -1647,7 +1647,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="81.75" customHeight="1">
+    <row r="101" ht="113.45" customHeight="1">
       <c r="A101" s="1" t="inlineStr">
         <is>
           <t>H199</t>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="81.75" customHeight="1">
+    <row r="102" ht="113.45" customHeight="1">
       <c r="A102" s="1" t="inlineStr">
         <is>
           <t>H201</t>
@@ -1671,7 +1671,7 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="81.75" customHeight="1">
+    <row r="103" ht="113.45" customHeight="1">
       <c r="A103" s="1" t="inlineStr">
         <is>
           <t>H203</t>
@@ -1683,7 +1683,7 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="81.75" customHeight="1">
+    <row r="104" ht="113.45" customHeight="1">
       <c r="A104" s="1" t="inlineStr">
         <is>
           <t>H205</t>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="81.75" customHeight="1">
+    <row r="105" ht="113.45" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
         <is>
           <t>H207</t>
@@ -1707,7 +1707,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="81.75" customHeight="1">
+    <row r="106" ht="113.45" customHeight="1">
       <c r="A106" s="1" t="inlineStr">
         <is>
           <t>H209</t>
@@ -1719,7 +1719,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="81.75" customHeight="1">
+    <row r="107" ht="113.45" customHeight="1">
       <c r="A107" s="1" t="inlineStr">
         <is>
           <t>H211</t>
@@ -1731,7 +1731,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="81.75" customHeight="1">
+    <row r="108" ht="113.45" customHeight="1">
       <c r="A108" s="1" t="inlineStr">
         <is>
           <t>H213</t>
@@ -1743,7 +1743,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="81.75" customHeight="1">
+    <row r="109" ht="113.45" customHeight="1">
       <c r="A109" s="1" t="inlineStr">
         <is>
           <t>H215</t>
@@ -1755,7 +1755,7 @@
         </is>
       </c>
     </row>
-    <row r="110" ht="81.75" customHeight="1">
+    <row r="110" ht="113.45" customHeight="1">
       <c r="A110" s="1" t="inlineStr">
         <is>
           <t>H217</t>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="81.75" customHeight="1">
+    <row r="111" ht="113.45" customHeight="1">
       <c r="A111" s="1" t="inlineStr">
         <is>
           <t>H219</t>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
     </row>
-    <row r="112" ht="81.75" customHeight="1">
+    <row r="112" ht="113.45" customHeight="1">
       <c r="A112" s="1" t="inlineStr">
         <is>
           <t>H221</t>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
     </row>
-    <row r="113" ht="81.75" customHeight="1">
+    <row r="113" ht="113.45" customHeight="1">
       <c r="A113" s="1" t="inlineStr">
         <is>
           <t>H223</t>
@@ -1803,7 +1803,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="81.75" customHeight="1">
+    <row r="114" ht="113.45" customHeight="1">
       <c r="A114" s="1" t="inlineStr">
         <is>
           <t>H225</t>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="81.75" customHeight="1">
+    <row r="115" ht="113.45" customHeight="1">
       <c r="A115" s="1" t="inlineStr">
         <is>
           <t>H227</t>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="81.75" customHeight="1">
+    <row r="116" ht="113.45" customHeight="1">
       <c r="A116" s="1" t="inlineStr">
         <is>
           <t>H229</t>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="81.75" customHeight="1">
+    <row r="117" ht="113.45" customHeight="1">
       <c r="A117" s="1" t="inlineStr">
         <is>
           <t>H231</t>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="81.75" customHeight="1">
+    <row r="118" ht="113.45" customHeight="1">
       <c r="A118" s="1" t="inlineStr">
         <is>
           <t>H233</t>
@@ -1863,7 +1863,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="81.75" customHeight="1">
+    <row r="119" ht="113.45" customHeight="1">
       <c r="A119" s="1" t="inlineStr">
         <is>
           <t>H235</t>
@@ -1875,7 +1875,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="81.75" customHeight="1">
+    <row r="120" ht="113.45" customHeight="1">
       <c r="A120" s="1" t="inlineStr">
         <is>
           <t>H237</t>
@@ -1887,7 +1887,7 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="81.75" customHeight="1">
+    <row r="121" ht="113.45" customHeight="1">
       <c r="A121" s="1" t="inlineStr">
         <is>
           <t>H239</t>
@@ -1899,7 +1899,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="81.75" customHeight="1">
+    <row r="122" ht="113.45" customHeight="1">
       <c r="A122" s="1" t="inlineStr">
         <is>
           <t>H241</t>
@@ -1911,7 +1911,7 @@
         </is>
       </c>
     </row>
-    <row r="123" ht="81.75" customHeight="1">
+    <row r="123" ht="113.45" customHeight="1">
       <c r="A123" s="1" t="inlineStr">
         <is>
           <t>H243</t>
@@ -1923,7 +1923,7 @@
         </is>
       </c>
     </row>
-    <row r="124" ht="81.75" customHeight="1">
+    <row r="124" ht="113.45" customHeight="1">
       <c r="A124" s="1" t="inlineStr">
         <is>
           <t>H245</t>
@@ -1935,7 +1935,7 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="81.75" customHeight="1">
+    <row r="125" ht="113.45" customHeight="1">
       <c r="A125" s="1" t="inlineStr">
         <is>
           <t>H247</t>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
     </row>
-    <row r="126" ht="81.75" customHeight="1">
+    <row r="126" ht="113.45" customHeight="1">
       <c r="A126" s="1" t="inlineStr">
         <is>
           <t>H249</t>
@@ -1959,7 +1959,7 @@
         </is>
       </c>
     </row>
-    <row r="127" ht="81.75" customHeight="1">
+    <row r="127" ht="113.45" customHeight="1">
       <c r="A127" s="1" t="inlineStr">
         <is>
           <t>H251</t>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
     </row>
-    <row r="128" ht="81.75" customHeight="1">
+    <row r="128" ht="113.45" customHeight="1">
       <c r="A128" s="1" t="inlineStr">
         <is>
           <t>H253</t>
@@ -1983,7 +1983,7 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="81.75" customHeight="1">
+    <row r="129" ht="113.45" customHeight="1">
       <c r="A129" s="1" t="inlineStr">
         <is>
           <t>H255</t>
@@ -1995,7 +1995,7 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="81.75" customHeight="1">
+    <row r="130" ht="113.45" customHeight="1">
       <c r="A130" s="1" t="inlineStr">
         <is>
           <t>H257</t>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="81.75" customHeight="1">
+    <row r="131" ht="113.45" customHeight="1">
       <c r="A131" s="1" t="inlineStr">
         <is>
           <t>H259</t>
@@ -2019,7 +2019,7 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="81.75" customHeight="1">
+    <row r="132" ht="113.45" customHeight="1">
       <c r="A132" s="1" t="inlineStr">
         <is>
           <t>H261</t>
@@ -2031,7 +2031,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="81.75" customHeight="1">
+    <row r="133" ht="113.45" customHeight="1">
       <c r="A133" s="1" t="inlineStr">
         <is>
           <t>H263</t>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
     </row>
-    <row r="134" ht="81.75" customHeight="1">
+    <row r="134" ht="113.45" customHeight="1">
       <c r="A134" s="1" t="inlineStr">
         <is>
           <t>H265</t>
@@ -2055,7 +2055,7 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="81.75" customHeight="1">
+    <row r="135" ht="113.45" customHeight="1">
       <c r="A135" s="1" t="inlineStr">
         <is>
           <t>H267</t>
@@ -2067,7 +2067,7 @@
         </is>
       </c>
     </row>
-    <row r="136" ht="81.75" customHeight="1">
+    <row r="136" ht="113.45" customHeight="1">
       <c r="A136" s="1" t="inlineStr">
         <is>
           <t>H269</t>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
     </row>
-    <row r="137" ht="81.75" customHeight="1">
+    <row r="137" ht="113.45" customHeight="1">
       <c r="A137" s="1" t="inlineStr">
         <is>
           <t>H271</t>
@@ -2091,7 +2091,7 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="81.75" customHeight="1">
+    <row r="138" ht="113.45" customHeight="1">
       <c r="A138" s="1" t="inlineStr">
         <is>
           <t>H273</t>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
     </row>
-    <row r="139" ht="81.75" customHeight="1">
+    <row r="139" ht="113.45" customHeight="1">
       <c r="A139" s="1" t="inlineStr">
         <is>
           <t>H275</t>
@@ -2115,7 +2115,7 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="81.75" customHeight="1">
+    <row r="140" ht="113.45" customHeight="1">
       <c r="A140" s="1" t="inlineStr">
         <is>
           <t>H277</t>
@@ -2127,7 +2127,7 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="81.75" customHeight="1">
+    <row r="141" ht="113.45" customHeight="1">
       <c r="A141" s="1" t="inlineStr">
         <is>
           <t>H279</t>
@@ -2139,7 +2139,7 @@
         </is>
       </c>
     </row>
-    <row r="142" ht="81.75" customHeight="1">
+    <row r="142" ht="113.45" customHeight="1">
       <c r="A142" s="1" t="inlineStr">
         <is>
           <t>H281</t>
@@ -2151,7 +2151,7 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="81.75" customHeight="1">
+    <row r="143" ht="113.45" customHeight="1">
       <c r="A143" s="1" t="inlineStr">
         <is>
           <t>H283</t>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
     </row>
-    <row r="144" ht="81.75" customHeight="1">
+    <row r="144" ht="113.45" customHeight="1">
       <c r="A144" s="1" t="inlineStr">
         <is>
           <t>H285</t>
@@ -2175,7 +2175,7 @@
         </is>
       </c>
     </row>
-    <row r="145" ht="81.75" customHeight="1">
+    <row r="145" ht="113.45" customHeight="1">
       <c r="A145" s="1" t="inlineStr">
         <is>
           <t>H287</t>
@@ -2186,7 +2186,7 @@
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup orientation="portrait" scale="78" fitToHeight="0"/>
-  <rowBreaks count="83" manualBreakCount="83">
+  <rowBreaks count="144" manualBreakCount="144">
     <brk id="1" min="0" max="16383" man="1"/>
     <brk id="2" min="0" max="16383" man="1"/>
     <brk id="3" min="0" max="16383" man="1"/>
@@ -2270,6 +2270,67 @@
     <brk id="81" min="0" max="16383" man="1"/>
     <brk id="82" min="0" max="16383" man="1"/>
     <brk id="83" min="0" max="16383" man="1"/>
+    <brk id="84" min="0" max="16383" man="1"/>
+    <brk id="85" min="0" max="16383" man="1"/>
+    <brk id="86" min="0" max="16383" man="1"/>
+    <brk id="87" min="0" max="16383" man="1"/>
+    <brk id="88" min="0" max="16383" man="1"/>
+    <brk id="89" min="0" max="16383" man="1"/>
+    <brk id="90" min="0" max="16383" man="1"/>
+    <brk id="91" min="0" max="16383" man="1"/>
+    <brk id="92" min="0" max="16383" man="1"/>
+    <brk id="93" min="0" max="16383" man="1"/>
+    <brk id="94" min="0" max="16383" man="1"/>
+    <brk id="95" min="0" max="16383" man="1"/>
+    <brk id="96" min="0" max="16383" man="1"/>
+    <brk id="97" min="0" max="16383" man="1"/>
+    <brk id="98" min="0" max="16383" man="1"/>
+    <brk id="99" min="0" max="16383" man="1"/>
+    <brk id="100" min="0" max="16383" man="1"/>
+    <brk id="101" min="0" max="16383" man="1"/>
+    <brk id="102" min="0" max="16383" man="1"/>
+    <brk id="103" min="0" max="16383" man="1"/>
+    <brk id="104" min="0" max="16383" man="1"/>
+    <brk id="105" min="0" max="16383" man="1"/>
+    <brk id="106" min="0" max="16383" man="1"/>
+    <brk id="107" min="0" max="16383" man="1"/>
+    <brk id="108" min="0" max="16383" man="1"/>
+    <brk id="109" min="0" max="16383" man="1"/>
+    <brk id="110" min="0" max="16383" man="1"/>
+    <brk id="111" min="0" max="16383" man="1"/>
+    <brk id="112" min="0" max="16383" man="1"/>
+    <brk id="113" min="0" max="16383" man="1"/>
+    <brk id="114" min="0" max="16383" man="1"/>
+    <brk id="115" min="0" max="16383" man="1"/>
+    <brk id="116" min="0" max="16383" man="1"/>
+    <brk id="117" min="0" max="16383" man="1"/>
+    <brk id="118" min="0" max="16383" man="1"/>
+    <brk id="119" min="0" max="16383" man="1"/>
+    <brk id="120" min="0" max="16383" man="1"/>
+    <brk id="121" min="0" max="16383" man="1"/>
+    <brk id="122" min="0" max="16383" man="1"/>
+    <brk id="123" min="0" max="16383" man="1"/>
+    <brk id="124" min="0" max="16383" man="1"/>
+    <brk id="125" min="0" max="16383" man="1"/>
+    <brk id="126" min="0" max="16383" man="1"/>
+    <brk id="127" min="0" max="16383" man="1"/>
+    <brk id="128" min="0" max="16383" man="1"/>
+    <brk id="129" min="0" max="16383" man="1"/>
+    <brk id="130" min="0" max="16383" man="1"/>
+    <brk id="131" min="0" max="16383" man="1"/>
+    <brk id="132" min="0" max="16383" man="1"/>
+    <brk id="133" min="0" max="16383" man="1"/>
+    <brk id="134" min="0" max="16383" man="1"/>
+    <brk id="135" min="0" max="16383" man="1"/>
+    <brk id="136" min="0" max="16383" man="1"/>
+    <brk id="137" min="0" max="16383" man="1"/>
+    <brk id="138" min="0" max="16383" man="1"/>
+    <brk id="139" min="0" max="16383" man="1"/>
+    <brk id="140" min="0" max="16383" man="1"/>
+    <brk id="141" min="0" max="16383" man="1"/>
+    <brk id="142" min="0" max="16383" man="1"/>
+    <brk id="143" min="0" max="16383" man="1"/>
+    <brk id="144" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>